<commit_message>
added new rule (wind spd >= 14)  in gust warning verification
</commit_message>
<xml_diff>
--- a/app/data/ad_warn_data/Aerodrome_Warnings_Table.xlsx
+++ b/app/data/ad_warn_data/Aerodrome_Warnings_Table.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Aerodrome Warnings" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aerodrome Warnings" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -442,7 +442,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Aerodrome warning for station VABB for 202601010003</t>
+          <t>Aerodrome warning for station VABB for July 2025</t>
         </is>
       </c>
     </row>
@@ -513,12 +513,12 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>nil</t>
+          <t>02/0600,02/1000,02/1400,06/0230,06/0645,14/0930,14/1330,14/1730,14/2130,15/0130,15/0530,21/0630,22/0430,22/0830,22/1200,22/1600,22/2000,23/0000,23/0400,25/0230,25/0600,25/1000,25/1400,26/1400,26/1800,26/2200</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>nil</t>
+          <t>96%</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -730,12 +730,12 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>30/0750,31/0530</t>
+          <t>01/0030,01/0430,01/0830,01/1230,01/1630,01/2030,02/0100,02/0500,02/0600,02/1000,02/1400,02/1800,02/2215,03/0200,03/0600,03/1000,03/1400,03/1630,03/2000,04/0040,04/0445,04/0830,04/1230,04/1630,04/2030,05/0030,05/0430,05/0830,05/1230,05/1700,05/2100,06/0100,06/0230,06/0645,06/1045,06/1430,06/1830,06/2230,07/0230,07/0630,07/1030,07/1430,07/1830,07/2230,08/0230,08/0645,08/1030,08/1430,08/1830,08/2230,09/0130,09/0530,09/0930,09/1530,09/1930,10/1030,10/1430,10/1930,11/0200,11/1000,12/0300,12/0700,12/1100,12/1500,12/1900,12/2300,13/0315,13/0715,13/1115,13/1915,14/0130,14/0530,14/0930,14/1330,14/1730,14/2130,15/0130,15/0530,15/0930,15/1330,15/1730,16/0630,16/1030,16/1430,17/0900,18/0745,18/1145,19/1000,20/0500,20/0900,20/1300,22/0800,22/1200,22/1600,22/2000,23/0000,23/0630,23/1030,23/1430,23/1900,24/0145,24/0600,24/1000,24/1400,24/1800,24/2200,25/0200,25/0600,25/1000,25/1400,25/1800,25/2200,26/0200,26/0600,26/1000,26/1400,26/1800,26/2200,27/0200,27/0600,27/1000,27/1400,27/1800,27/2100,28/0100,28/0500,28/0900,28/1345,28/1730,28/2130,29/0130,29/0530,29/0930,29/1330,29/1730,29/2130,30/0130,30/0530,30/0930,30/1330,30/1730,30/2130,31/0130,31/0530,31/1030,31/1445,31/1900,31/2300</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>81%</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">

</xml_diff>